<commit_message>
seed: align word-map enums and import locally
</commit_message>
<xml_diff>
--- a/docs/implementation/seed-data/canonical-spelling-word-map/canonical-spelling-word-map-v1.xlsx
+++ b/docs/implementation/seed-data/canonical-spelling-word-map/canonical-spelling-word-map-v1.xlsx
@@ -3631,7 +3631,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>contrast_practice</t>
+          <t>grouped_set_practice</t>
         </is>
       </c>
       <c r="J58" s="2" t="b">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>contrast_practice</t>
+          <t>grouped_set_practice</t>
         </is>
       </c>
       <c r="J59" s="2" t="b">
@@ -4181,7 +4181,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>contrast_practice</t>
+          <t>grouped_set_practice</t>
         </is>
       </c>
       <c r="J68" s="2" t="b">
@@ -4236,7 +4236,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>contrast_practice</t>
+          <t>grouped_set_practice</t>
         </is>
       </c>
       <c r="J69" s="2" t="b">
@@ -4731,7 +4731,7 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>contrast_practice</t>
+          <t>grouped_set_practice</t>
         </is>
       </c>
       <c r="J78" s="2" t="b">
@@ -4786,7 +4786,7 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>contrast_practice</t>
+          <t>grouped_set_practice</t>
         </is>
       </c>
       <c r="J79" s="2" t="b">
@@ -5281,7 +5281,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>contrast_practice</t>
+          <t>grouped_set_practice</t>
         </is>
       </c>
       <c r="J88" s="2" t="b">
@@ -5336,7 +5336,7 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>contrast_practice</t>
+          <t>grouped_set_practice</t>
         </is>
       </c>
       <c r="J89" s="2" t="b">
@@ -8344,7 +8344,7 @@
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I2" s="2" t="n">
@@ -8386,7 +8386,7 @@
       <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I3" s="2" t="n">
@@ -8428,7 +8428,7 @@
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I4" s="2" t="n">
@@ -8470,7 +8470,7 @@
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I5" s="2" t="n">
@@ -8512,7 +8512,7 @@
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I6" s="2" t="n">
@@ -8554,7 +8554,7 @@
       <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I7" s="2" t="n">
@@ -8596,7 +8596,7 @@
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I8" s="2" t="n">
@@ -8638,7 +8638,7 @@
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>partly_irregular</t>
         </is>
       </c>
       <c r="I9" s="2" t="n">
@@ -8680,7 +8680,7 @@
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I10" s="2" t="n">
@@ -8722,7 +8722,7 @@
       <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I11" s="2" t="n">
@@ -8764,7 +8764,7 @@
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I12" s="2" t="n">
@@ -8806,7 +8806,7 @@
       <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I13" s="2" t="n">
@@ -8848,7 +8848,7 @@
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I14" s="2" t="n">
@@ -8890,7 +8890,7 @@
       <c r="G15" s="2" t="inlineStr"/>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I15" s="2" t="n">
@@ -8932,7 +8932,7 @@
       <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I16" s="2" t="n">
@@ -8974,7 +8974,7 @@
       <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I17" s="2" t="n">
@@ -9016,7 +9016,7 @@
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
@@ -9058,7 +9058,7 @@
       <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I19" s="2" t="n">
@@ -9100,7 +9100,7 @@
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
@@ -9142,7 +9142,7 @@
       <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I21" s="2" t="n">
@@ -9184,7 +9184,7 @@
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I22" s="2" t="n">
@@ -9226,7 +9226,7 @@
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I23" s="2" t="n">
@@ -9268,7 +9268,7 @@
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
@@ -9310,7 +9310,7 @@
       <c r="G25" s="2" t="inlineStr"/>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I25" s="2" t="n">
@@ -9352,7 +9352,7 @@
       <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I26" s="2" t="n">
@@ -9394,7 +9394,7 @@
       <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I27" s="2" t="n">
@@ -9436,7 +9436,7 @@
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I28" s="2" t="n">
@@ -9478,7 +9478,7 @@
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I29" s="2" t="n">
@@ -9520,7 +9520,7 @@
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I30" s="2" t="n">
@@ -9562,7 +9562,7 @@
       <c r="G31" s="2" t="inlineStr"/>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I31" s="2" t="n">
@@ -9604,7 +9604,7 @@
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I32" s="2" t="n">
@@ -9646,7 +9646,7 @@
       <c r="G33" s="2" t="inlineStr"/>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I33" s="2" t="n">
@@ -9688,7 +9688,7 @@
       <c r="G34" s="2" t="inlineStr"/>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I34" s="2" t="n">
@@ -9730,7 +9730,7 @@
       <c r="G35" s="2" t="inlineStr"/>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I35" s="2" t="n">
@@ -9772,7 +9772,7 @@
       <c r="G36" s="2" t="inlineStr"/>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>partly_irregular</t>
         </is>
       </c>
       <c r="I36" s="2" t="n">
@@ -9814,7 +9814,7 @@
       <c r="G37" s="2" t="inlineStr"/>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I37" s="2" t="n">
@@ -9856,7 +9856,7 @@
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I38" s="2" t="n">
@@ -9898,7 +9898,7 @@
       <c r="G39" s="2" t="inlineStr"/>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I39" s="2" t="n">
@@ -9940,7 +9940,7 @@
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I40" s="2" t="n">
@@ -9982,7 +9982,7 @@
       <c r="G41" s="2" t="inlineStr"/>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I41" s="2" t="n">
@@ -10024,7 +10024,7 @@
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>partly_irregular</t>
         </is>
       </c>
       <c r="I42" s="2" t="n">
@@ -10066,7 +10066,7 @@
       <c r="G43" s="2" t="inlineStr"/>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I43" s="2" t="n">
@@ -10108,7 +10108,7 @@
       <c r="G44" s="2" t="inlineStr"/>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I44" s="2" t="n">
@@ -10150,7 +10150,7 @@
       <c r="G45" s="2" t="inlineStr"/>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>partly_irregular</t>
         </is>
       </c>
       <c r="I45" s="2" t="n">
@@ -10192,7 +10192,7 @@
       <c r="G46" s="2" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I46" s="2" t="n">
@@ -10234,7 +10234,7 @@
       <c r="G47" s="2" t="inlineStr"/>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I47" s="2" t="n">
@@ -10276,7 +10276,7 @@
       <c r="G48" s="2" t="inlineStr"/>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I48" s="2" t="n">
@@ -10318,7 +10318,7 @@
       <c r="G49" s="2" t="inlineStr"/>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I49" s="2" t="n">
@@ -10360,7 +10360,7 @@
       <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I50" s="2" t="n">
@@ -10402,7 +10402,7 @@
       <c r="G51" s="2" t="inlineStr"/>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I51" s="2" t="n">
@@ -10444,7 +10444,7 @@
       <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I52" s="2" t="n">
@@ -10486,7 +10486,7 @@
       <c r="G53" s="2" t="inlineStr"/>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I53" s="2" t="n">
@@ -10528,7 +10528,7 @@
       <c r="G54" s="2" t="inlineStr"/>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I54" s="2" t="n">
@@ -10570,7 +10570,7 @@
       <c r="G55" s="2" t="inlineStr"/>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I55" s="2" t="n">
@@ -10612,7 +10612,7 @@
       <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I56" s="2" t="n">
@@ -10654,7 +10654,7 @@
       <c r="G57" s="2" t="inlineStr"/>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I57" s="2" t="n">
@@ -10696,7 +10696,7 @@
       <c r="G58" s="2" t="inlineStr"/>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I58" s="2" t="n">
@@ -10738,7 +10738,7 @@
       <c r="G59" s="2" t="inlineStr"/>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I59" s="2" t="n">
@@ -10780,7 +10780,7 @@
       <c r="G60" s="2" t="inlineStr"/>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I60" s="2" t="n">
@@ -10822,7 +10822,7 @@
       <c r="G61" s="2" t="inlineStr"/>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I61" s="2" t="n">
@@ -10864,7 +10864,7 @@
       <c r="G62" s="2" t="inlineStr"/>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I62" s="2" t="n">
@@ -10906,7 +10906,7 @@
       <c r="G63" s="2" t="inlineStr"/>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I63" s="2" t="n">
@@ -10948,7 +10948,7 @@
       <c r="G64" s="2" t="inlineStr"/>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I64" s="2" t="n">
@@ -10990,7 +10990,7 @@
       <c r="G65" s="2" t="inlineStr"/>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I65" s="2" t="n">
@@ -11032,7 +11032,7 @@
       <c r="G66" s="2" t="inlineStr"/>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I66" s="2" t="n">
@@ -11074,7 +11074,7 @@
       <c r="G67" s="2" t="inlineStr"/>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I67" s="2" t="n">
@@ -11116,7 +11116,7 @@
       <c r="G68" s="2" t="inlineStr"/>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I68" s="2" t="n">
@@ -11158,7 +11158,7 @@
       <c r="G69" s="2" t="inlineStr"/>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I69" s="2" t="n">
@@ -11200,7 +11200,7 @@
       <c r="G70" s="2" t="inlineStr"/>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I70" s="2" t="n">
@@ -11242,7 +11242,7 @@
       <c r="G71" s="2" t="inlineStr"/>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>partly_irregular</t>
         </is>
       </c>
       <c r="I71" s="2" t="n">
@@ -11284,7 +11284,7 @@
       <c r="G72" s="2" t="inlineStr"/>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I72" s="2" t="n">
@@ -11326,7 +11326,7 @@
       <c r="G73" s="2" t="inlineStr"/>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I73" s="2" t="n">
@@ -11368,7 +11368,7 @@
       <c r="G74" s="2" t="inlineStr"/>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I74" s="2" t="n">
@@ -11410,7 +11410,7 @@
       <c r="G75" s="2" t="inlineStr"/>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I75" s="2" t="n">
@@ -11452,7 +11452,7 @@
       <c r="G76" s="2" t="inlineStr"/>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I76" s="2" t="n">
@@ -11494,7 +11494,7 @@
       <c r="G77" s="2" t="inlineStr"/>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I77" s="2" t="n">
@@ -11536,7 +11536,7 @@
       <c r="G78" s="2" t="inlineStr"/>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I78" s="2" t="n">
@@ -11578,7 +11578,7 @@
       <c r="G79" s="2" t="inlineStr"/>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I79" s="2" t="n">
@@ -11620,7 +11620,7 @@
       <c r="G80" s="2" t="inlineStr"/>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I80" s="2" t="n">
@@ -11662,7 +11662,7 @@
       <c r="G81" s="2" t="inlineStr"/>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I81" s="2" t="n">
@@ -11704,7 +11704,7 @@
       <c r="G82" s="2" t="inlineStr"/>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I82" s="2" t="n">
@@ -11746,7 +11746,7 @@
       <c r="G83" s="2" t="inlineStr"/>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I83" s="2" t="n">
@@ -11788,7 +11788,7 @@
       <c r="G84" s="2" t="inlineStr"/>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I84" s="2" t="n">
@@ -11830,7 +11830,7 @@
       <c r="G85" s="2" t="inlineStr"/>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I85" s="2" t="n">
@@ -11872,7 +11872,7 @@
       <c r="G86" s="2" t="inlineStr"/>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I86" s="2" t="n">
@@ -11914,7 +11914,7 @@
       <c r="G87" s="2" t="inlineStr"/>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I87" s="2" t="n">
@@ -11956,7 +11956,7 @@
       <c r="G88" s="2" t="inlineStr"/>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I88" s="2" t="n">
@@ -11998,7 +11998,7 @@
       <c r="G89" s="2" t="inlineStr"/>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I89" s="2" t="n">
@@ -12040,7 +12040,7 @@
       <c r="G90" s="2" t="inlineStr"/>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I90" s="2" t="n">
@@ -12082,7 +12082,7 @@
       <c r="G91" s="2" t="inlineStr"/>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I91" s="2" t="n">
@@ -12124,7 +12124,7 @@
       <c r="G92" s="2" t="inlineStr"/>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>partly_irregular</t>
         </is>
       </c>
       <c r="I92" s="2" t="n">
@@ -12166,7 +12166,7 @@
       <c r="G93" s="2" t="inlineStr"/>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I93" s="2" t="n">
@@ -12208,7 +12208,7 @@
       <c r="G94" s="2" t="inlineStr"/>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I94" s="2" t="n">
@@ -12250,7 +12250,7 @@
       <c r="G95" s="2" t="inlineStr"/>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I95" s="2" t="n">
@@ -12292,7 +12292,7 @@
       <c r="G96" s="2" t="inlineStr"/>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I96" s="2" t="n">
@@ -12334,7 +12334,7 @@
       <c r="G97" s="2" t="inlineStr"/>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I97" s="2" t="n">
@@ -12376,7 +12376,7 @@
       <c r="G98" s="2" t="inlineStr"/>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I98" s="2" t="n">
@@ -12418,7 +12418,7 @@
       <c r="G99" s="2" t="inlineStr"/>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I99" s="2" t="n">
@@ -12460,7 +12460,7 @@
       <c r="G100" s="2" t="inlineStr"/>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="I100" s="2" t="n">
@@ -12483,7 +12483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -13075,23 +13075,23 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>D4_PG_LONG_AI_FINAL_AY</t>
+          <t>D4_PG_LONG_AI_MEDIAL_AI</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>contrast_practice</t>
+          <t>word_practice</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D23" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>spelling_contrast_v1</t>
+          <t>spelling_word_practice_v1</t>
         </is>
       </c>
       <c r="F23" s="2" t="b">
@@ -13106,7 +13106,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>word_practice</t>
+          <t>grouped_set_practice</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -13117,7 +13117,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>spelling_word_practice_v1</t>
+          <t>spelling_grouped_set_v1</t>
         </is>
       </c>
       <c r="F24" s="2" t="b">
@@ -13132,18 +13132,18 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>grouped_set_practice</t>
+          <t>dictation</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D25" s="2" t="b">
         <v>0</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>spelling_grouped_set_v1</t>
+          <t>spelling_dictation_v1</t>
         </is>
       </c>
       <c r="F25" s="2" t="b">
@@ -13153,23 +13153,23 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>D4_PG_LONG_AI_MEDIAL_AI</t>
+          <t>D4_PG_LONG_OA_OA</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>dictation</t>
+          <t>word_practice</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D26" s="2" t="b">
         <v>0</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>spelling_dictation_v1</t>
+          <t>spelling_word_practice_v1</t>
         </is>
       </c>
       <c r="F26" s="2" t="b">
@@ -13179,23 +13179,23 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>D4_PG_LONG_AI_MEDIAL_AI</t>
+          <t>D4_PG_LONG_OA_OA</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>contrast_practice</t>
+          <t>grouped_set_practice</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D27" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>spelling_contrast_v1</t>
+          <t>spelling_grouped_set_v1</t>
         </is>
       </c>
       <c r="F27" s="2" t="b">
@@ -13210,18 +13210,18 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>word_practice</t>
+          <t>dictation</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D28" s="2" t="b">
         <v>0</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>spelling_word_practice_v1</t>
+          <t>spelling_dictation_v1</t>
         </is>
       </c>
       <c r="F28" s="2" t="b">
@@ -13231,12 +13231,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>D4_PG_LONG_OA_OA</t>
+          <t>D4_PAT_SPLIT_DIGRAPHS_A_E</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>grouped_set_practice</t>
+          <t>word_practice</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -13247,7 +13247,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>spelling_grouped_set_v1</t>
+          <t>spelling_word_practice_v1</t>
         </is>
       </c>
       <c r="F29" s="2" t="b">
@@ -13257,23 +13257,23 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>D4_PG_LONG_OA_OA</t>
+          <t>D4_PAT_SPLIT_DIGRAPHS_A_E</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>dictation</t>
+          <t>grouped_set_practice</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D30" s="2" t="b">
         <v>0</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>spelling_dictation_v1</t>
+          <t>spelling_grouped_set_v1</t>
         </is>
       </c>
       <c r="F30" s="2" t="b">
@@ -13283,130 +13283,26 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>D4_PG_LONG_OA_OA</t>
+          <t>D4_PAT_SPLIT_DIGRAPHS_A_E</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>contrast_practice</t>
+          <t>dictation</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D31" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>spelling_contrast_v1</t>
+          <t>spelling_dictation_v1</t>
         </is>
       </c>
       <c r="F31" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>D4_PAT_SPLIT_DIGRAPHS_A_E</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>word_practice</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D32" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>spelling_word_practice_v1</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>D4_PAT_SPLIT_DIGRAPHS_A_E</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>grouped_set_practice</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D33" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>spelling_grouped_set_v1</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>D4_PAT_SPLIT_DIGRAPHS_A_E</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>dictation</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D34" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>spelling_dictation_v1</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>D4_PAT_SPLIT_DIGRAPHS_A_E</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>contrast_practice</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D35" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>spelling_contrast_v1</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>